<commit_message>
Add DrHall ECMR3 QA repair pipeline
Introduce DrHall ECMR3 QA hallucination-repair pipeline (gpt-4o/drhall.py). The new script implements a 3-stage ECMR3 flow: generate k paraphrases of the question, verify-and-repair the base answer per paraphrase path, and perform semantic-consistency majority voting to produce a single final_answer. It includes a safe_chat_call wrapper, paraphrase extraction, resume/save logic, token/time logging, and writes outputs to ./outputs/{model}_drhall_ecmr3_{dataset}.csv (default model: gpt-4o).

Also add three new prompts to gpt-4o/llm_prompts/prompts.py: PARAPHRASE_PROMPT_DRHALL_QA, REPAIR_PROMPT_DRHALL_QA, and CONSISTENCY_VOTE_PROMPT_DRHALL_QA. Updated stat/leetcode.xlsx (binary diff).
</commit_message>
<xml_diff>
--- a/stat/leetcode.xlsx
+++ b/stat/leetcode.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr\Documents\Workspace\LLMHalluMiti\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{919F83F3-4612-4142-82E3-025457558EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0DECD74-58FA-4E6D-9049-703370225B7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{311A53CD-DEC1-4332-A976-671472767E86}"/>
   </bookViews>
@@ -91,7 +91,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -107,16 +107,51 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -124,23 +159,74 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -471,427 +557,440 @@
     <col min="10" max="10" width="20.625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C1" t="s">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A1" s="2"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="4">
         <v>130</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="5">
         <f>C2/200</f>
         <v>0.65</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="4">
         <v>124</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="5">
         <f>E2/200</f>
         <v>0.62</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="4">
         <v>6</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="5">
         <f>G2/C2</f>
         <v>4.6153846153846156E-2</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="6">
         <v>0</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="7">
         <f>I2/(200-C2)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B3" t="s">
+    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="2"/>
+      <c r="B3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="8">
         <v>130</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="9">
         <f t="shared" ref="D3:D13" si="0">C3/200</f>
         <v>0.65</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="8">
         <v>127</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="9">
         <f t="shared" ref="F3:F13" si="1">E3/200</f>
         <v>0.63500000000000001</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="8">
         <v>4</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="9">
         <f>G3/C3</f>
         <v>3.0769230769230771E-2</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="8">
         <v>1</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="9">
         <f>I3/(200-C3)</f>
         <v>1.4285714285714285E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B4" t="s">
+    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="2"/>
+      <c r="B4" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="12">
         <v>130</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="13">
         <f t="shared" si="0"/>
         <v>0.65</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="14">
         <v>102</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="15">
         <f t="shared" si="1"/>
         <v>0.51</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="14">
         <v>30</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="15">
         <f t="shared" ref="H4:H13" si="2">G4/C4</f>
         <v>0.23076923076923078</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="12">
         <v>3</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="13">
         <f>I4/(200-C4)</f>
         <v>4.2857142857142858E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+    <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="4">
         <v>53</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="5">
         <f t="shared" si="0"/>
         <v>0.26500000000000001</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="4">
         <v>44</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="5">
         <f t="shared" si="1"/>
         <v>0.22</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="4">
         <v>10</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="5">
         <f t="shared" si="2"/>
         <v>0.18867924528301888</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="4">
         <v>1</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="5">
         <f t="shared" ref="J5:J13" si="3">I5/(200-C5)</f>
         <v>6.8027210884353739E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B6" t="s">
+    <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A6" s="2"/>
+      <c r="B6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="8">
         <v>53</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="9">
         <f t="shared" si="0"/>
         <v>0.26500000000000001</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="8">
         <v>47</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="9">
         <f t="shared" si="1"/>
         <v>0.23499999999999999</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="8">
         <v>6</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="9">
         <f t="shared" si="2"/>
         <v>0.11320754716981132</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="8">
         <v>0</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="9">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B7" t="s">
+    <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A7" s="2"/>
+      <c r="B7" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="12">
         <v>53</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="13">
         <f t="shared" si="0"/>
         <v>0.26500000000000001</v>
       </c>
-      <c r="F7" s="1">
+      <c r="E7" s="12"/>
+      <c r="F7" s="13">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H7" s="1">
+      <c r="G7" s="12"/>
+      <c r="H7" s="13">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J7" s="1">
+      <c r="I7" s="12"/>
+      <c r="J7" s="13">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="8" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="4">
         <v>97</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="5">
         <f t="shared" si="0"/>
         <v>0.48499999999999999</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="4">
         <v>87</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="5">
         <f t="shared" si="1"/>
         <v>0.435</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="4">
         <v>12</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="5">
         <f t="shared" si="2"/>
         <v>0.12371134020618557</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="6">
         <v>2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="7">
         <f t="shared" si="3"/>
         <v>1.9417475728155338E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B9" t="s">
+    <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A9" s="2"/>
+      <c r="B9" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="8">
         <v>97</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="9">
         <f t="shared" si="0"/>
         <v>0.48499999999999999</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="8">
         <v>62</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="9">
         <f t="shared" si="1"/>
         <v>0.31</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="8">
         <v>37</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="9">
         <f t="shared" si="2"/>
         <v>0.38144329896907214</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="10">
         <v>2</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="11">
         <f t="shared" si="3"/>
         <v>1.9417475728155338E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B10" t="s">
+    <row r="10" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A10" s="2"/>
+      <c r="B10" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="12">
         <v>97</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="13">
         <f t="shared" si="0"/>
         <v>0.48499999999999999</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="14">
         <v>58</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="15">
         <f t="shared" si="1"/>
         <v>0.28999999999999998</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="14">
         <v>41</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="15">
         <f t="shared" si="2"/>
         <v>0.42268041237113402</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="14">
         <v>2</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="15">
         <f t="shared" si="3"/>
         <v>1.9417475728155338E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+    <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="4">
         <v>158</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="5">
         <f t="shared" si="0"/>
         <v>0.79</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="4">
         <v>157</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11" s="5">
         <f t="shared" si="1"/>
         <v>0.78500000000000003</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="4">
         <v>7</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="5">
         <f t="shared" si="2"/>
         <v>4.4303797468354431E-2</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="4">
         <v>6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="5">
         <f t="shared" si="3"/>
         <v>0.14285714285714285</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B12" t="s">
+    <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A12" s="2"/>
+      <c r="B12" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="8">
         <v>158</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="9">
         <f t="shared" si="0"/>
         <v>0.79</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="8">
         <v>151</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12" s="9">
         <f t="shared" si="1"/>
         <v>0.755</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="8">
         <v>7</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="9">
         <f t="shared" si="2"/>
         <v>4.4303797468354431E-2</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="10">
         <v>0</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="11">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B13" t="s">
+    <row r="13" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A13" s="2"/>
+      <c r="B13" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="12">
         <v>158</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="13">
         <f t="shared" si="0"/>
         <v>0.79</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="14">
         <v>90</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13" s="15">
         <f t="shared" si="1"/>
         <v>0.45</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="14">
         <v>71</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="15">
         <f t="shared" si="2"/>
         <v>0.44936708860759494</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="12">
         <v>3</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="13">
         <f t="shared" si="3"/>
         <v>7.1428571428571425E-2</v>
       </c>

</xml_diff>

<commit_message>
Update evaluation results, metrics and outputs
Rename evaluation run to gpt-5_mutrepair and adjust final pass flags in evaluation_results.csv (several tasks changed from False->True and a few True->False). Update evaluation_results.metrics.json with revised counts and metrics (n_final_hall, n_repaired, n_over_corrected, HR/RHR/HRR/OCR). Normalize numeric fields in gpt-5_mutrepair_gpt-5_leetcode_responses.csv (integers converted to floats with .0) and append/replace multiple candidate implementations—notably many variants of minimizedMaximum and sumPrefixScores, plus other mutation artifacts—into the responses CSV. Also update stat/leetcode.xlsx (spreadsheet updated). These changes reflect a new mutation-repair evaluation run and result formatting adjustments.
</commit_message>
<xml_diff>
--- a/stat/leetcode.xlsx
+++ b/stat/leetcode.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr\Documents\Workspace\LLMHalluMiti\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0DECD74-58FA-4E6D-9049-703370225B7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F734C71D-D774-4A1D-B885-A24F2437AFF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{311A53CD-DEC1-4332-A976-671472767E86}"/>
   </bookViews>
@@ -151,7 +151,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -174,13 +174,159 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -190,21 +336,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -227,6 +358,69 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -557,440 +751,446 @@
     <col min="10" max="10" width="20.625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A1" s="2"/>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2" t="s">
+    <row r="1" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="11"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="27" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="16">
         <v>130</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="17">
         <f>C2/200</f>
         <v>0.65</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="16">
         <v>124</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="17">
         <f>E2/200</f>
         <v>0.62</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="16">
         <v>6</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="17">
         <f>G2/C2</f>
         <v>4.6153846153846156E-2</v>
       </c>
-      <c r="I2" s="6">
+      <c r="I2" s="28">
         <v>0</v>
       </c>
-      <c r="J2" s="7">
+      <c r="J2" s="29">
         <f>I2/(200-C2)</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="2"/>
-      <c r="B3" s="8" t="s">
+      <c r="A3" s="19"/>
+      <c r="B3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="3">
         <v>130</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="4">
         <f t="shared" ref="D3:D13" si="0">C3/200</f>
         <v>0.65</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="3">
         <v>127</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="4">
         <f t="shared" ref="F3:F13" si="1">E3/200</f>
         <v>0.63500000000000001</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="3">
         <v>4</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="4">
         <f>G3/C3</f>
         <v>3.0769230769230771E-2</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="3">
         <v>1</v>
       </c>
-      <c r="J3" s="9">
+      <c r="J3" s="30">
         <f>I3/(200-C3)</f>
         <v>1.4285714285714285E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="2"/>
-      <c r="B4" s="12" t="s">
+    <row r="4" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="21"/>
+      <c r="B4" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="22">
         <v>130</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="23">
         <f t="shared" si="0"/>
         <v>0.65</v>
       </c>
-      <c r="E4" s="14">
+      <c r="E4" s="24">
         <v>102</v>
       </c>
-      <c r="F4" s="15">
+      <c r="F4" s="25">
         <f t="shared" si="1"/>
         <v>0.51</v>
       </c>
-      <c r="G4" s="14">
+      <c r="G4" s="24">
         <v>30</v>
       </c>
-      <c r="H4" s="15">
+      <c r="H4" s="25">
         <f t="shared" ref="H4:H13" si="2">G4/C4</f>
         <v>0.23076923076923078</v>
       </c>
-      <c r="I4" s="12">
+      <c r="I4" s="22">
         <v>3</v>
       </c>
-      <c r="J4" s="13">
+      <c r="J4" s="26">
         <f>I4/(200-C4)</f>
         <v>4.2857142857142858E-2</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="16">
         <v>53</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="17">
         <f t="shared" si="0"/>
         <v>0.26500000000000001</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="16">
         <v>44</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="17">
         <f t="shared" si="1"/>
         <v>0.22</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="16">
         <v>10</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="17">
         <f t="shared" si="2"/>
         <v>0.18867924528301888</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="16">
         <v>1</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="18">
         <f t="shared" ref="J5:J13" si="3">I5/(200-C5)</f>
         <v>6.8027210884353739E-3</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="2"/>
-      <c r="B6" s="8" t="s">
+      <c r="A6" s="19"/>
+      <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="3">
         <v>53</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="4">
         <f t="shared" si="0"/>
         <v>0.26500000000000001</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="3">
         <v>47</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="4">
         <f t="shared" si="1"/>
         <v>0.23499999999999999</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="3">
         <v>6</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H6" s="4">
         <f t="shared" si="2"/>
         <v>0.11320754716981132</v>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="5">
         <v>0</v>
       </c>
-      <c r="J6" s="9">
+      <c r="J6" s="20">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="2"/>
-      <c r="B7" s="12" t="s">
+    <row r="7" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="21"/>
+      <c r="B7" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="22">
         <v>53</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="23">
         <f t="shared" si="0"/>
         <v>0.26500000000000001</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="13">
+      <c r="E7" s="24">
+        <v>41</v>
+      </c>
+      <c r="F7" s="25">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G7" s="12"/>
-      <c r="H7" s="13">
+        <v>0.20499999999999999</v>
+      </c>
+      <c r="G7" s="24">
+        <v>14</v>
+      </c>
+      <c r="H7" s="25">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I7" s="12"/>
-      <c r="J7" s="13">
+        <v>0.26415094339622641</v>
+      </c>
+      <c r="I7" s="22">
+        <v>2</v>
+      </c>
+      <c r="J7" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.3605442176870748E-2</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="16">
         <v>97</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="17">
         <f t="shared" si="0"/>
         <v>0.48499999999999999</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="16">
         <v>87</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="17">
         <f t="shared" si="1"/>
         <v>0.435</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="16">
         <v>12</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="17">
         <f t="shared" si="2"/>
         <v>0.12371134020618557</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="28">
         <v>2</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="29">
         <f t="shared" si="3"/>
         <v>1.9417475728155338E-2</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="2"/>
-      <c r="B9" s="8" t="s">
+      <c r="A9" s="19"/>
+      <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="3">
         <v>97</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="4">
         <f t="shared" si="0"/>
         <v>0.48499999999999999</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="3">
         <v>62</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="4">
         <f t="shared" si="1"/>
         <v>0.31</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="3">
         <v>37</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="4">
         <f t="shared" si="2"/>
         <v>0.38144329896907214</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I9" s="5">
         <v>2</v>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="20">
         <f t="shared" si="3"/>
         <v>1.9417475728155338E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="2"/>
-      <c r="B10" s="12" t="s">
+    <row r="10" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="21"/>
+      <c r="B10" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="22">
         <v>97</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="23">
         <f t="shared" si="0"/>
         <v>0.48499999999999999</v>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="24">
         <v>58</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="25">
         <f t="shared" si="1"/>
         <v>0.28999999999999998</v>
       </c>
-      <c r="G10" s="14">
+      <c r="G10" s="24">
         <v>41</v>
       </c>
-      <c r="H10" s="15">
+      <c r="H10" s="25">
         <f t="shared" si="2"/>
         <v>0.42268041237113402</v>
       </c>
-      <c r="I10" s="14">
+      <c r="I10" s="24">
         <v>2</v>
       </c>
-      <c r="J10" s="15">
+      <c r="J10" s="31">
         <f t="shared" si="3"/>
         <v>1.9417475728155338E-2</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="13">
         <v>158</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="14">
         <f t="shared" si="0"/>
         <v>0.79</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="13">
         <v>157</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="14">
         <f t="shared" si="1"/>
         <v>0.78500000000000003</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="13">
         <v>7</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="14">
         <f t="shared" si="2"/>
         <v>4.4303797468354431E-2</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I11" s="13">
         <v>6</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="14">
         <f t="shared" si="3"/>
         <v>0.14285714285714285</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="3">
         <v>158</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="4">
         <f t="shared" si="0"/>
         <v>0.79</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="3">
         <v>151</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="4">
         <f t="shared" si="1"/>
         <v>0.755</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="3">
         <v>7</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H12" s="4">
         <f t="shared" si="2"/>
         <v>4.4303797468354431E-2</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="5">
         <v>0</v>
       </c>
-      <c r="J12" s="11">
+      <c r="J12" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="12">
+      <c r="C13" s="7">
         <v>158</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="8">
         <f t="shared" si="0"/>
         <v>0.79</v>
       </c>
-      <c r="E13" s="14">
+      <c r="E13" s="9">
         <v>90</v>
       </c>
-      <c r="F13" s="15">
+      <c r="F13" s="10">
         <f t="shared" si="1"/>
         <v>0.45</v>
       </c>
-      <c r="G13" s="14">
+      <c r="G13" s="9">
         <v>71</v>
       </c>
-      <c r="H13" s="15">
+      <c r="H13" s="10">
         <f t="shared" si="2"/>
         <v>0.44936708860759494</v>
       </c>
-      <c r="I13" s="12">
+      <c r="I13" s="7">
         <v>3</v>
       </c>
-      <c r="J13" s="13">
+      <c r="J13" s="8">
         <f t="shared" si="3"/>
         <v>7.1428571428571425E-2</v>
       </c>

</xml_diff>